<commit_message>
Document folder update: - chaned IO Port_Usage_Planning.xls - new information regarding KTY81 - textfile with usefuls links
</commit_message>
<xml_diff>
--- a/Documents/Port_Usage_Planning.xlsx
+++ b/Documents/Port_Usage_Planning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bekone01-my.sharepoint.com/personal/juergen_eggeling_beko-technologies_com/Documents/_Projekte/_Bastelprojekte/SaunaControlUnit/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juerg\Documents\_Workspaces\SaunaControlUnit\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{E941FA22-BFF3-459E-889C-BA1D0C939ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A52A154C-65FC-471F-A41E-ED115C467187}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8F4052-6FE0-4303-B2E7-8CCF809AEBBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32220" yWindow="3420" windowWidth="38700" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33450" yWindow="-5280" windowWidth="28800" windowHeight="20480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signal view" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="151">
   <si>
     <t>Funktion</t>
   </si>
@@ -486,10 +486,7 @@
     <t>ESP module connector view</t>
   </si>
   <si>
-    <t>Debug_1</t>
-  </si>
-  <si>
-    <t>Debug_2</t>
+    <t>Debug</t>
   </si>
 </sst>
 </file>
@@ -1033,13 +1030,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
@@ -1692,31 +1689,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="20" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="66" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="66" t="s">
+      <c r="H1" s="68" t="s">
         <v>128</v>
       </c>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
-      <c r="O1" s="66" t="s">
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="O1" s="68" t="s">
         <v>129</v>
       </c>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="68"/>
     </row>
     <row r="2" spans="1:20" ht="29.5" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
@@ -3036,7 +3033,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9221DBC-EDCA-460E-9237-EA76481AB5F0}">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="6.6328125" style="1" customWidth="1"/>
@@ -3051,40 +3048,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="20" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="66" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
     </row>
     <row r="2" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:13" ht="20" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="67" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="H3" s="66" t="s">
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="H3" s="68" t="s">
         <v>129</v>
       </c>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
     </row>
     <row r="4" spans="1:13" s="65" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A4" s="18" t="s">
@@ -3191,7 +3188,7 @@
         <v>35</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="L6" s="11" t="s">
         <v>14</v>
@@ -3629,22 +3626,18 @@
       <c r="F18" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="21">
         <v>14</v>
       </c>
-      <c r="I18" s="54" t="s">
+      <c r="I18" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="J18" s="54" t="s">
-        <v>35</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="M18" s="24" t="s">
+      <c r="J18" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="22" t="s">
         <v>84</v>
       </c>
     </row>
@@ -3667,22 +3660,22 @@
       <c r="F19" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="H19" s="27">
+      <c r="H19" s="23">
         <v>16</v>
       </c>
-      <c r="I19" s="53" t="s">
+      <c r="I19" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="J19" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="K19" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="L19" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="M19" s="28" t="s">
+      <c r="J19" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="M19" s="24" t="s">
         <v>86</v>
       </c>
     </row>
@@ -3839,6 +3832,26 @@
       <c r="K26" s="70"/>
       <c r="L26" s="70"/>
       <c r="M26" s="70"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="H28" s="27">
+        <v>16</v>
+      </c>
+      <c r="I28" s="53" t="s">
+        <v>85</v>
+      </c>
+      <c r="J28" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="M28" s="28" t="s">
+        <v>86</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Remarks to port usage added
</commit_message>
<xml_diff>
--- a/Documents/Port_Usage_Planning.xlsx
+++ b/Documents/Port_Usage_Planning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juerg\Documents\_Workspaces\SaunaControlUnit\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8F4052-6FE0-4303-B2E7-8CCF809AEBBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2D1B3F-F7B0-4453-9C04-60F9A64BAC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33450" yWindow="-5280" windowWidth="28800" windowHeight="20480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25680" yWindow="-4110" windowWidth="27240" windowHeight="17030" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signal view" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="155">
   <si>
     <t>Funktion</t>
   </si>
@@ -487,6 +487,18 @@
   </si>
   <si>
     <t>Debug</t>
+  </si>
+  <si>
+    <t>Light on/ff</t>
+  </si>
+  <si>
+    <t>Mode</t>
+  </si>
+  <si>
+    <t>GPIO2, ADC2_CH2, TOUCH_CH2, !!!)</t>
+  </si>
+  <si>
+    <t>!!!) If KTY not connected (Uin 3,3V) System does not enter Boot mode properly!</t>
   </si>
 </sst>
 </file>
@@ -857,7 +869,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1080,6 +1092,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3033,775 +3054,797 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9221DBC-EDCA-460E-9237-EA76481AB5F0}">
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="6.6328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.08984375" customWidth="1"/>
+    <col min="1" max="1" width="3.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="39.7265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.54296875" customWidth="1"/>
-    <col min="8" max="10" width="6.6328125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.54296875" customWidth="1"/>
-    <col min="12" max="12" width="14.26953125" customWidth="1"/>
+    <col min="8" max="8" width="3.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="34.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="20" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="83" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
-    </row>
-    <row r="2" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:13" ht="20" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="67" t="s">
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+    </row>
+    <row r="2" spans="1:13" ht="20.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="67" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="H3" s="68" t="s">
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="H2" s="68" t="s">
         <v>129</v>
       </c>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-    </row>
-    <row r="4" spans="1:13" s="65" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="18" t="s">
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+    </row>
+    <row r="3" spans="1:13" s="65" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="63" t="s">
+      <c r="B3" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="63" t="s">
+      <c r="C3" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="63" t="s">
+      <c r="D3" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="63" t="s">
+      <c r="E3" s="63" t="s">
         <v>145</v>
       </c>
-      <c r="F4" s="64" t="s">
+      <c r="F3" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="H3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="63" t="s">
+      <c r="I3" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="63" t="s">
+      <c r="J3" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="K4" s="63" t="s">
+      <c r="K3" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="63" t="s">
+      <c r="L3" s="63" t="s">
         <v>145</v>
       </c>
-      <c r="M4" s="64" t="s">
+      <c r="M3" s="64" t="s">
         <v>146</v>
       </c>
     </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="59">
+        <v>1</v>
+      </c>
+      <c r="B4" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="F4" s="62" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="59">
+        <v>1</v>
+      </c>
+      <c r="I4" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="60" t="s">
+        <v>137</v>
+      </c>
+      <c r="K4" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="L4" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="M4" s="62" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="59">
+      <c r="A5" s="36">
+        <v>2</v>
+      </c>
+      <c r="B5" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E5" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="F5" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="27">
+        <v>2</v>
+      </c>
+      <c r="I5" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="L5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="M5" s="28" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="23">
+        <v>3</v>
+      </c>
+      <c r="B6" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="60" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="E5" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="F5" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="59">
-        <v>1</v>
-      </c>
-      <c r="I5" s="60" t="s">
-        <v>49</v>
-      </c>
-      <c r="J5" s="60" t="s">
-        <v>137</v>
-      </c>
-      <c r="K5" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="L5" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="M5" s="62" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="21">
-        <v>2</v>
-      </c>
-      <c r="B6" s="51" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="51" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F6" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="27">
-        <v>2</v>
-      </c>
-      <c r="I6" s="53" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="L6" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="M6" s="28" t="s">
-        <v>63</v>
+      <c r="E6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="34">
+        <v>3</v>
+      </c>
+      <c r="I6" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="M6" s="35" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B7" s="54" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" s="54" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="34">
-        <v>3</v>
-      </c>
-      <c r="I7" s="52" t="s">
-        <v>64</v>
-      </c>
-      <c r="J7" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="K7" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="L7" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="M7" s="35" t="s">
-        <v>110</v>
+        <v>29</v>
+      </c>
+      <c r="H7" s="36">
+        <v>4</v>
+      </c>
+      <c r="I7" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="J7" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="37"/>
+      <c r="L7" s="37"/>
+      <c r="M7" s="39" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" s="54" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" s="54" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="H8" s="21">
-        <v>4</v>
-      </c>
-      <c r="I8" s="51" t="s">
-        <v>66</v>
-      </c>
-      <c r="J8" s="51" t="s">
-        <v>35</v>
-      </c>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="22" t="s">
-        <v>67</v>
+        <v>31</v>
+      </c>
+      <c r="H8" s="36">
+        <v>5</v>
+      </c>
+      <c r="I8" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+      <c r="M8" s="39" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" s="54" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C9" s="54" t="s">
         <v>24</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="21">
+        <v>33</v>
+      </c>
+      <c r="H9" s="34">
+        <v>6</v>
+      </c>
+      <c r="I9" s="52" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="M9" s="35" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="25">
+        <v>7</v>
+      </c>
+      <c r="B10" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="57" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="51" t="s">
-        <v>68</v>
-      </c>
-      <c r="J9" s="51" t="s">
-        <v>35</v>
-      </c>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="22" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="23">
-        <v>6</v>
-      </c>
-      <c r="B10" s="54" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="54" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="H10" s="34">
-        <v>6</v>
-      </c>
-      <c r="I10" s="52" t="s">
-        <v>70</v>
-      </c>
-      <c r="J10" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="L10" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="M10" s="35" t="s">
-        <v>111</v>
+      <c r="E10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="59">
+        <v>7</v>
+      </c>
+      <c r="I10" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="J10" s="60" t="s">
+        <v>137</v>
+      </c>
+      <c r="K10" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="L10" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="M10" s="62" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="25">
+        <v>8</v>
+      </c>
+      <c r="B11" s="57" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>7</v>
-      </c>
-      <c r="B11" s="57" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>5</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="59">
-        <v>7</v>
-      </c>
-      <c r="I11" s="60" t="s">
-        <v>49</v>
-      </c>
-      <c r="J11" s="60" t="s">
-        <v>137</v>
-      </c>
-      <c r="K11" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="L11" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="M11" s="62" t="s">
-        <v>51</v>
+        <v>38</v>
+      </c>
+      <c r="H11" s="27">
+        <v>8</v>
+      </c>
+      <c r="I11" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="M11" s="28" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="25">
+        <v>9</v>
+      </c>
+      <c r="B12" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="57" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>8</v>
-      </c>
-      <c r="B12" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>7</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="27">
-        <v>8</v>
-      </c>
-      <c r="I12" s="53" t="s">
-        <v>71</v>
-      </c>
-      <c r="J12" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="K12" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="L12" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="M12" s="28" t="s">
-        <v>72</v>
+        <v>40</v>
+      </c>
+      <c r="H12" s="43">
+        <v>9</v>
+      </c>
+      <c r="I12" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M12" s="29" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="25">
+      <c r="A13" s="27">
+        <v>10</v>
+      </c>
+      <c r="B13" s="53" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="57" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>40</v>
+      <c r="E13" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>42</v>
       </c>
       <c r="H13" s="43">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I13" s="47" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J13" s="47" t="s">
         <v>35</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>13</v>
       </c>
       <c r="M13" s="29" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="27">
+        <v>11</v>
+      </c>
+      <c r="B14" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>10</v>
-      </c>
-      <c r="B14" s="53" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>9</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>132</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H14" s="43">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I14" s="47" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J14" s="47" t="s">
         <v>35</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L14" s="9" t="s">
         <v>13</v>
       </c>
       <c r="M14" s="29" t="s">
-        <v>76</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="27">
+        <v>12</v>
+      </c>
+      <c r="B15" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>11</v>
-      </c>
-      <c r="B15" s="53" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>10</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>132</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="H15" s="43">
-        <v>11</v>
-      </c>
-      <c r="I15" s="47" t="s">
-        <v>77</v>
-      </c>
-      <c r="J15" s="47" t="s">
-        <v>35</v>
-      </c>
-      <c r="K15" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="L15" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="H15" s="27">
+        <v>12</v>
+      </c>
+      <c r="I15" s="53" t="s">
+        <v>79</v>
+      </c>
+      <c r="J15" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="M15" s="28" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" s="25">
         <v>13</v>
       </c>
-      <c r="M15" s="29" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="27">
+      <c r="B16" s="57" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="57" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="23">
+        <v>13</v>
+      </c>
+      <c r="I16" s="54" t="s">
+        <v>81</v>
+      </c>
+      <c r="J16" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="L16" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="53" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F16" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="H16" s="27">
+      <c r="M16" s="24" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" s="59">
+        <v>14</v>
+      </c>
+      <c r="B17" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="60" t="s">
+        <v>137</v>
+      </c>
+      <c r="D17" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="F17" s="62" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" s="21">
+        <v>14</v>
+      </c>
+      <c r="I17" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="J17" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" s="25">
+        <v>15</v>
+      </c>
+      <c r="B18" s="57" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="57" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="H18" s="23">
+        <v>16</v>
+      </c>
+      <c r="I18" s="54" t="s">
+        <v>85</v>
+      </c>
+      <c r="J18" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="L18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="53" t="s">
-        <v>79</v>
-      </c>
-      <c r="J16" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="K16" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="M16" s="28" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A17" s="25">
+      <c r="M18" s="85" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" s="36">
+        <v>16</v>
+      </c>
+      <c r="B19" s="55" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="71" t="s">
+        <v>144</v>
+      </c>
+      <c r="E19" s="72"/>
+      <c r="F19" s="73"/>
+      <c r="H19" s="43">
+        <v>17</v>
+      </c>
+      <c r="I19" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="J19" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="L19" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="57" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="H17" s="23">
-        <v>13</v>
-      </c>
-      <c r="I17" s="54" t="s">
-        <v>81</v>
-      </c>
-      <c r="J17" s="54" t="s">
-        <v>35</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="L17" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="M17" s="24" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A18" s="59">
-        <v>14</v>
-      </c>
-      <c r="B18" s="60" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="60" t="s">
-        <v>137</v>
-      </c>
-      <c r="D18" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="E18" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="F18" s="62" t="s">
-        <v>51</v>
-      </c>
-      <c r="H18" s="21">
-        <v>14</v>
-      </c>
-      <c r="I18" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="J18" s="51" t="s">
-        <v>35</v>
-      </c>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="22" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A19" s="25">
-        <v>15</v>
-      </c>
-      <c r="B19" s="57" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="H19" s="23">
-        <v>16</v>
-      </c>
-      <c r="I19" s="54" t="s">
-        <v>85</v>
-      </c>
-      <c r="J19" s="54" t="s">
-        <v>35</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="L19" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="M19" s="24" t="s">
-        <v>86</v>
+      <c r="M19" s="29" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="36">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="55" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C20" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="71" t="s">
+      <c r="D20" s="74"/>
+      <c r="E20" s="75"/>
+      <c r="F20" s="76"/>
+      <c r="H20" s="36">
+        <v>17</v>
+      </c>
+      <c r="I20" s="55" t="s">
+        <v>89</v>
+      </c>
+      <c r="J20" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="K20" s="71" t="s">
         <v>144</v>
       </c>
-      <c r="E20" s="72"/>
-      <c r="F20" s="73"/>
-      <c r="H20" s="43">
-        <v>17</v>
-      </c>
-      <c r="I20" s="47" t="s">
-        <v>87</v>
-      </c>
-      <c r="J20" s="47" t="s">
-        <v>35</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="L20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="M20" s="29" t="s">
-        <v>88</v>
-      </c>
+      <c r="L20" s="72"/>
+      <c r="M20" s="73"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="36">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="55" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C21" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="75"/>
-      <c r="F21" s="76"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="79"/>
       <c r="H21" s="36">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I21" s="55" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J21" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="K21" s="71" t="s">
-        <v>144</v>
-      </c>
-      <c r="L21" s="72"/>
-      <c r="M21" s="73"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A22" s="36">
-        <v>18</v>
-      </c>
-      <c r="B22" s="55" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" s="55" t="s">
-        <v>35</v>
-      </c>
-      <c r="D22" s="77"/>
-      <c r="E22" s="78"/>
-      <c r="F22" s="79"/>
-      <c r="H22" s="36">
-        <v>18</v>
-      </c>
-      <c r="I22" s="55" t="s">
-        <v>91</v>
-      </c>
-      <c r="J22" s="55" t="s">
-        <v>35</v>
-      </c>
-      <c r="K22" s="74"/>
-      <c r="L22" s="75"/>
-      <c r="M22" s="76"/>
-    </row>
-    <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="59">
+      <c r="K21" s="74"/>
+      <c r="L21" s="75"/>
+      <c r="M21" s="76"/>
+    </row>
+    <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="59">
         <v>19</v>
       </c>
-      <c r="B23" s="60" t="s">
+      <c r="B22" s="60" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="60" t="s">
+      <c r="C22" s="60" t="s">
         <v>137</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D22" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E22" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="F23" s="62" t="s">
+      <c r="F22" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="H23" s="40">
+      <c r="H22" s="40">
         <v>19</v>
       </c>
-      <c r="I23" s="56" t="s">
+      <c r="I22" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="J23" s="56" t="s">
-        <v>35</v>
-      </c>
-      <c r="K23" s="80"/>
-      <c r="L23" s="81"/>
-      <c r="M23" s="82"/>
+      <c r="J22" s="56" t="s">
+        <v>35</v>
+      </c>
+      <c r="K22" s="80"/>
+      <c r="L22" s="81"/>
+      <c r="M22" s="82"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" s="84" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="44"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="75" t="s">
+        <v>154</v>
+      </c>
+      <c r="I24" s="75"/>
+      <c r="J24" s="75"/>
+      <c r="K24" s="75"/>
+      <c r="L24" s="75"/>
+      <c r="M24" s="75"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="69" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B25" s="70"/>
       <c r="C25" s="70"/>
@@ -3816,58 +3859,22 @@
       <c r="L25" s="70"/>
       <c r="M25" s="70"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A26" s="69" t="s">
-        <v>117</v>
-      </c>
-      <c r="B26" s="70"/>
-      <c r="C26" s="70"/>
-      <c r="D26" s="70"/>
-      <c r="E26" s="70"/>
-      <c r="F26" s="70"/>
-      <c r="G26" s="70"/>
-      <c r="H26" s="70"/>
-      <c r="I26" s="70"/>
-      <c r="J26" s="70"/>
-      <c r="K26" s="70"/>
-      <c r="L26" s="70"/>
-      <c r="M26" s="70"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="H28" s="27">
-        <v>16</v>
-      </c>
-      <c r="I28" s="53" t="s">
-        <v>85</v>
-      </c>
-      <c r="J28" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="K28" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="L28" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="M28" s="28" t="s">
-        <v>86</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="H3:M3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="H2:M2"/>
     <mergeCell ref="A25:M25"/>
-    <mergeCell ref="A26:M26"/>
-    <mergeCell ref="D20:F22"/>
-    <mergeCell ref="K21:M23"/>
+    <mergeCell ref="D19:F21"/>
+    <mergeCell ref="K20:M22"/>
+    <mergeCell ref="H24:M24"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A26" r:id="rId1" xr:uid="{8C29EB1E-5FC7-4B4B-B6D2-9EF086296AB7}"/>
-    <hyperlink ref="A25" r:id="rId2" xr:uid="{66CDB618-6607-4CC0-9408-30BF1EA62DE2}"/>
+    <hyperlink ref="A25" r:id="rId1" xr:uid="{8C29EB1E-5FC7-4B4B-B6D2-9EF086296AB7}"/>
+    <hyperlink ref="A24" r:id="rId2" xr:uid="{66CDB618-6607-4CC0-9408-30BF1EA62DE2}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>